<commit_message>
Update test cases and data files for improved accuracy and clarity; remove unnecessary cache files
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Enter Marks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GPA" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,12 +30,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -56,11 +62,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -137,25 +143,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TestCases" displayName="TestCases" ref="A1:J23" headerRowCount="1">
-  <autoFilter ref="A1:J23"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="TC ID"/>
-    <tableColumn id="2" name="Module"/>
-    <tableColumn id="3" name="Function"/>
-    <tableColumn id="4" name="Technique"/>
-    <tableColumn id="5" name="Description"/>
-    <tableColumn id="6" name="Precondition"/>
-    <tableColumn id="7" name="Test Data"/>
-    <tableColumn id="8" name="Expected Result"/>
-    <tableColumn id="9" name="Data Source (tests/data/)"/>
-    <tableColumn id="10" name="Status"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,19 +434,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,45 +454,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Module</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Function</t>
+          <t>Precondition</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Technique</t>
+          <t>Test Data</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Precondition</t>
+          <t>Actual Result</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Data Source (tests/data/)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -517,50 +486,37 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-01</t>
+          <t>TC-EM-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Highest possible marks</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 100</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lowest valid marks</t>
+          <t>Grade A</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=0</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Grade F, 0.0 points</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -569,50 +525,37 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-02</t>
+          <t>TC-EM-02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Middle of the A band</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 92</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Just below the D boundary</t>
+          <t>Grade A</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=49.99</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Grade F, 0.0 points</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -621,50 +564,37 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-03</t>
+          <t>TC-EM-03</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Lowest marks for A</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 85</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>On the D boundary</t>
+          <t>Grade A</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=50</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Grade D, 1.0 points</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
+          <t>Grade A</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -673,50 +603,37 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-04</t>
+          <t>TC-EM-04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Just below the A boundary</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 84.99</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nominal C+ marks</t>
+          <t>Grade A-</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=62</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Grade C+, 2.3 points</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
+          <t>Grade A-</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -725,50 +642,37 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-05</t>
+          <t>TC-EM-05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Middle of the A- band</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 82</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Just below the A boundary</t>
+          <t>Grade A-</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=84.99</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Grade A-, 3.7 points</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
+          <t>Grade A-</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -777,50 +681,37 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-06</t>
+          <t>TC-EM-06</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Lowest marks for A-</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 80</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On the A boundary</t>
+          <t>Grade A-</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=85</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Grade A, 4.0 points</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+          <t>Grade A-</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -829,50 +720,37 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-07</t>
+          <t>TC-EM-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Just below the A- boundary</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 79.99</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Highest valid marks</t>
+          <t>Grade B+</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=100</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Grade A, 4.0 points</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+          <t>Grade B+</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -881,50 +759,37 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-08</t>
+          <t>TC-EM-08</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Middle of the B+ band</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 77</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Just below zero</t>
+          <t>Grade B+</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=-0.01</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Raises ValueError</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+          <t>Grade B+</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -933,50 +798,37 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-09</t>
+          <t>TC-EM-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Lowest marks for B+</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 75</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Just above 100</t>
+          <t>Grade B+</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=100.01</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Raises ValueError</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
+          <t>Grade B+</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -985,50 +837,37 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-10</t>
+          <t>TC-EM-10</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Just below the B+ boundary</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 74.99</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Far out of range</t>
+          <t>Grade B</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=CS101, marks=250</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Raises ValueError</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1037,50 +876,37 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-11</t>
+          <t>TC-EM-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Middle of the B band</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 72</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Unknown student</t>
+          <t>Grade B</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-999, code=CS101, marks=75</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Raises KeyError</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1089,50 +915,37 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TC-DD-12</t>
+          <t>TC-EM-12</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>sms.school</t>
+          <t>Lowest marks for B</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>School.enter_marks</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 70</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Course the student is not enrolled in</t>
+          <t>Grade B</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Student CS-001 enrolled in CS101 (marks 90)</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>roll_no=CS-001, code=AI201, marks=75</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Raises KeyError</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>enter_marks_cases.csv</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
+          <t>Grade B</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1141,50 +954,37 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-01</t>
+          <t>TC-EM-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Just below the B boundary</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 69.99</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>No courses</t>
+          <t>Grade B-</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>marks=[none], credits=[none]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>GPA 0.0</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1193,50 +993,37 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-02</t>
+          <t>TC-EM-14</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Middle of the B- band</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 67</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>One A course</t>
+          <t>Grade B-</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>marks=[90], credits=[3]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>GPA 4.0</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1245,50 +1032,37 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-03</t>
+          <t>TC-EM-15</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Lowest marks for B-</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 65</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>All courses F (minimum GPA)</t>
+          <t>Grade B-</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>marks=[10;49.99], credits=[3;4]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>GPA 0.0</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
+          <t>Grade B-</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1297,50 +1071,37 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-04</t>
+          <t>TC-EM-16</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Just below the B- boundary</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 64.99</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>All courses on the A boundary (maximum GPA)</t>
+          <t>Grade C+</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>marks=[85;100], credits=[3;4]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>GPA 4.0</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
+          <t>Grade C+</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1349,50 +1110,37 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-05</t>
+          <t>TC-EM-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Middle of the C+ band</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 62</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Weighted by credit hours</t>
+          <t>Grade C+</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>marks=[90;72], credits=[3;2]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>GPA 3.6</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
+          <t>Grade C+</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1401,50 +1149,37 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-06</t>
+          <t>TC-EM-18</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Lowest marks for C+</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 60</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Weighted with an F</t>
+          <t>Grade C+</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>marks=[90;72;49], credits=[3;2;4]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>GPA 2.0</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
+          <t>Grade C+</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1453,50 +1188,37 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-07</t>
+          <t>TC-EM-19</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Just below the C+ boundary</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 59.99</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Result rounded to 2 decimals (12/7)</t>
+          <t>Grade C</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>marks=[90;49], credits=[3;4]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>GPA 1.71</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
+          <t>Grade C</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1505,50 +1227,37 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-08</t>
+          <t>TC-EM-20</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Middle of the C band</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 57</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Ungraded course ignored</t>
+          <t>Grade C</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>marks=[90;-], credits=[3;4]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>GPA 4.0</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
+          <t>Grade C</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1557,50 +1266,37 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-09</t>
+          <t>TC-EM-21</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Lowest marks for C</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ECP</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 55</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>All courses ungraded</t>
+          <t>Grade C</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>marks=[-;-], credits=[3;2]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>GPA 0.0</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
+          <t>Grade C</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1609,50 +1305,583 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TC-GPA-10</t>
+          <t>TC-EM-22</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>sms.grading</t>
+          <t>Just below the C boundary</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>calculate_gpa</t>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>BVA</t>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 54.99</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Lower boundaries of A / A- / B+</t>
+          <t>Grade D</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>marks=[85;80;75], credits=[1;1;1]  ('-' = not entered)</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>GPA 3.67</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>gpa_cases.csv</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
+          <t>Grade D</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Middle of the D band</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 52</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Grade D</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Grade D</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Lowest marks for D (pass mark)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 50</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Grade D</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Grade D</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Just below the pass mark</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 49.99</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Grade F</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Grade F</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Middle of the F band</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 25</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Grade F</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Grade F</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Lowest possible marks</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 0</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Grade F</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Grade F</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>First marks for a course that had no marks yet</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: EN101
+Marks: 81</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Grade A-</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Grade A-</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Just below 0</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: -0.01</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Negative marks</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: -10</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Just above 100</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 100.01</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Far above 100</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: CS101
+Marks: 150</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Error: marks must be between 0 and 100 (ValueError)</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Student does not exist</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-999
+Course: CS101
+Marks: 75</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Roll no in lowercase</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: cs-001
+Course: CS101
+Marks: 75</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Course code in lowercase</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: cs101
+Marks: 75</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-EM-36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Student is not enrolled in the course</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Student CS-001 is enrolled in CS101 (marks 90) and EN101 (no marks yet)</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Roll no: CS-001
+Course: AI201
+Marks: 75</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Error: student or course not found (KeyError)</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -1660,8 +1889,597 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Both courses A: (4.0x3 + 4.0x3) / 6</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 90, 3 credits
+Course 2: marks 95, 3 credits</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>GPA 4.0</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>GPA 4.0</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Both courses F: (0x3 + 0x3) / 6</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 30, 3 credits
+Course 2: marks 45, 3 credits</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.0</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.0</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>A and B with different credits: (4.0x3 + 3.0x2) / 5</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 90, 3 credits
+Course 2: marks 72, 2 credits</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>GPA 3.6</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>GPA 3.6</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>A and F rounded to 2 decimals: (4.0x3 + 0x4) / 7 = 1.714</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 90, 3 credits
+Course 2: marks 40, 4 credits</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>GPA 1.71</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>GPA 1.71</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Boundary marks A and A-: (4.0x3 + 3.7x3) / 6</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 85, 3 credits
+Course 2: marks 84.99, 3 credits</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>GPA 3.85</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>GPA 3.85</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>A- and B+: (3.7x3 + 3.3x3) / 6</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 82, 3 credits
+Course 2: marks 77, 3 credits</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>GPA 3.5</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>GPA 3.5</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>B and B-: (3.0x2 + 2.7x2) / 4</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 72, 2 credits
+Course 2: marks 67, 2 credits</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>GPA 2.85</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>GPA 2.85</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>C+ and C: (2.3x3 + 2.0x2) / 5</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 62, 3 credits
+Course 2: marks 57, 2 credits</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>GPA 2.18</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>GPA 2.18</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Boundary marks D and F: (1.0x3 + 0x3) / 6</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 50, 3 credits
+Course 2: marks 49.99, 3 credits</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.5</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.5</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>C and D rounded to 2 decimals: (2.0x2 + 1.0x4) / 6 = 1.333</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 55, 2 credits
+Course 2: marks 52, 4 credits</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>GPA 1.33</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>GPA 1.33</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Highest and lowest marks: (4.0x3 + 0x3) / 6</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 100, 3 credits
+Course 2: marks 0, 3 credits</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>GPA 2.0</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>GPA 2.0</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Course with more credits counts more: (4.0x1 + 0x5) / 6 = 0.667</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 90, 1 credits
+Course 2: marks 40, 5 credits</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.67</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.67</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Second course has no marks yet so it is ignored: (4.0x3) / 3</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: marks 90, 3 credits
+Course 2: no marks yet, 4 credits</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>GPA 4.0</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>GPA 4.0</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-GPA-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>No marks entered for either course</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Course 1: no marks yet, 3 credits
+Course 2: no marks yet, 2 credits</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.0</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>GPA 0.0</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>